<commit_message>
Complete draft-day remediation on main.
Promote hardened sale/ESPN paths, ME-gated My Roster formulas, HQ layout/contrast fixes, and launch preflight so tonight's auction runs from verified main.
</commit_message>
<xml_diff>
--- a/Draft_Command_Center_DRAFT_DAY.xlsx
+++ b/Draft_Command_Center_DRAFT_DAY.xlsx
@@ -3213,6 +3213,9 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <color rgb="FF1A1A1A"/>
+      </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFF2CC"/>
@@ -3244,6 +3247,9 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <color rgb="FF1A1A1A"/>
+      </font>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFC6EFCE"/>
@@ -3395,6 +3401,9 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <color rgb="FF1A1A1A"/>
+      </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
@@ -3759,6 +3768,9 @@
       </border>
     </dxf>
     <dxf>
+      <font>
+        <color rgb="FF1A1A1A"/>
+      </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFF2CC"/>
@@ -3773,6 +3785,9 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <color rgb="FF1A1A1A"/>
+      </font>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFFF2CC"/>
@@ -3808,6 +3823,9 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <color rgb="FF1A1A1A"/>
+      </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFF2CC"/>
@@ -4952,18 +4970,19 @@
   <dimension ref="A1:N38"/>
   <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="1" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.0"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10.0"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="5.0"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12.0"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="13.0"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="9.0"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="14.0"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="10.0"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="7.0"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="9.0"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="9.0"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="11.0"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="13.0"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="18"/>
   </cols>
   <sheetData>
@@ -44155,7 +44174,7 @@
         <v>16</v>
       </c>
       <c r="B7" s="15" t="str">
-        <f aca="false">IFERROR(INDEX('Auction Log'!$B$5:$B$304,MATCH(A7,'Auction Log'!$F$5:$F$304,0)),"")</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Auction Log'!$F$5:$F$304=A7)*('Auction Log'!$D$5:$D$304="ME")),'Auction Log'!$B$5:$B$304),"")</f>
         <v/>
       </c>
       <c r="C7" s="15" t="str">
@@ -44163,7 +44182,7 @@
         <v/>
       </c>
       <c r="D7" s="16" t="str">
-        <f aca="false">IFERROR(INDEX('Auction Log'!$E$5:$E$304,MATCH(A7,'Auction Log'!$F$5:$F$304,0)),"")</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Auction Log'!$F$5:$F$304=A7)*('Auction Log'!$D$5:$D$304="ME")),'Auction Log'!$E$5:$E$304),"")</f>
         <v/>
       </c>
       <c r="E7" s="15" t="str">
@@ -44196,7 +44215,7 @@
         <v>503</v>
       </c>
       <c r="B8" s="18" t="str">
-        <f aca="false">IFERROR(INDEX('Auction Log'!$B$5:$B$304,MATCH(A8,'Auction Log'!$F$5:$F$304,0)),"")</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Auction Log'!$F$5:$F$304=A8)*('Auction Log'!$D$5:$D$304="ME")),'Auction Log'!$B$5:$B$304),"")</f>
         <v/>
       </c>
       <c r="C8" s="18" t="str">
@@ -44204,7 +44223,7 @@
         <v/>
       </c>
       <c r="D8" s="19" t="str">
-        <f aca="false">IFERROR(INDEX('Auction Log'!$E$5:$E$304,MATCH(A8,'Auction Log'!$F$5:$F$304,0)),"")</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Auction Log'!$F$5:$F$304=A8)*('Auction Log'!$D$5:$D$304="ME")),'Auction Log'!$E$5:$E$304),"")</f>
         <v/>
       </c>
       <c r="E8" s="18" t="str">
@@ -44237,7 +44256,7 @@
         <v>504</v>
       </c>
       <c r="B9" s="18" t="str">
-        <f aca="false">IFERROR(INDEX('Auction Log'!$B$5:$B$304,MATCH(A9,'Auction Log'!$F$5:$F$304,0)),"")</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Auction Log'!$F$5:$F$304=A9)*('Auction Log'!$D$5:$D$304="ME")),'Auction Log'!$B$5:$B$304),"")</f>
         <v/>
       </c>
       <c r="C9" s="18" t="str">
@@ -44245,7 +44264,7 @@
         <v/>
       </c>
       <c r="D9" s="19" t="str">
-        <f aca="false">IFERROR(INDEX('Auction Log'!$E$5:$E$304,MATCH(A9,'Auction Log'!$F$5:$F$304,0)),"")</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Auction Log'!$F$5:$F$304=A9)*('Auction Log'!$D$5:$D$304="ME")),'Auction Log'!$E$5:$E$304),"")</f>
         <v/>
       </c>
       <c r="E9" s="18" t="str">
@@ -44278,7 +44297,7 @@
         <v>505</v>
       </c>
       <c r="B10" s="18" t="str">
-        <f aca="false">IFERROR(INDEX('Auction Log'!$B$5:$B$304,MATCH(A10,'Auction Log'!$F$5:$F$304,0)),"")</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Auction Log'!$F$5:$F$304=A10)*('Auction Log'!$D$5:$D$304="ME")),'Auction Log'!$B$5:$B$304),"")</f>
         <v/>
       </c>
       <c r="C10" s="18" t="str">
@@ -44286,7 +44305,7 @@
         <v/>
       </c>
       <c r="D10" s="19" t="str">
-        <f aca="false">IFERROR(INDEX('Auction Log'!$E$5:$E$304,MATCH(A10,'Auction Log'!$F$5:$F$304,0)),"")</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Auction Log'!$F$5:$F$304=A10)*('Auction Log'!$D$5:$D$304="ME")),'Auction Log'!$E$5:$E$304),"")</f>
         <v/>
       </c>
       <c r="E10" s="18" t="str">
@@ -44319,7 +44338,7 @@
         <v>506</v>
       </c>
       <c r="B11" s="18" t="str">
-        <f aca="false">IFERROR(INDEX('Auction Log'!$B$5:$B$304,MATCH(A11,'Auction Log'!$F$5:$F$304,0)),"")</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Auction Log'!$F$5:$F$304=A11)*('Auction Log'!$D$5:$D$304="ME")),'Auction Log'!$B$5:$B$304),"")</f>
         <v/>
       </c>
       <c r="C11" s="18" t="str">
@@ -44327,7 +44346,7 @@
         <v/>
       </c>
       <c r="D11" s="19" t="str">
-        <f aca="false">IFERROR(INDEX('Auction Log'!$E$5:$E$304,MATCH(A11,'Auction Log'!$F$5:$F$304,0)),"")</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Auction Log'!$F$5:$F$304=A11)*('Auction Log'!$D$5:$D$304="ME")),'Auction Log'!$E$5:$E$304),"")</f>
         <v/>
       </c>
       <c r="E11" s="18" t="str">
@@ -44360,7 +44379,7 @@
         <v>30</v>
       </c>
       <c r="B12" s="18" t="str">
-        <f aca="false">IFERROR(INDEX('Auction Log'!$B$5:$B$304,MATCH(A12,'Auction Log'!$F$5:$F$304,0)),"")</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Auction Log'!$F$5:$F$304=A12)*('Auction Log'!$D$5:$D$304="ME")),'Auction Log'!$B$5:$B$304),"")</f>
         <v/>
       </c>
       <c r="C12" s="18" t="str">
@@ -44368,7 +44387,7 @@
         <v/>
       </c>
       <c r="D12" s="19" t="str">
-        <f aca="false">IFERROR(INDEX('Auction Log'!$E$5:$E$304,MATCH(A12,'Auction Log'!$F$5:$F$304,0)),"")</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Auction Log'!$F$5:$F$304=A12)*('Auction Log'!$D$5:$D$304="ME")),'Auction Log'!$E$5:$E$304),"")</f>
         <v/>
       </c>
       <c r="E12" s="18" t="str">
@@ -44401,7 +44420,7 @@
         <v>507</v>
       </c>
       <c r="B13" s="18" t="str">
-        <f aca="false">IFERROR(INDEX('Auction Log'!$B$5:$B$304,MATCH(A13,'Auction Log'!$F$5:$F$304,0)),"")</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Auction Log'!$F$5:$F$304=A13)*('Auction Log'!$D$5:$D$304="ME")),'Auction Log'!$B$5:$B$304),"")</f>
         <v/>
       </c>
       <c r="C13" s="18" t="str">
@@ -44409,7 +44428,7 @@
         <v/>
       </c>
       <c r="D13" s="19" t="str">
-        <f aca="false">IFERROR(INDEX('Auction Log'!$E$5:$E$304,MATCH(A13,'Auction Log'!$F$5:$F$304,0)),"")</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Auction Log'!$F$5:$F$304=A13)*('Auction Log'!$D$5:$D$304="ME")),'Auction Log'!$E$5:$E$304),"")</f>
         <v/>
       </c>
       <c r="E13" s="18" t="str">
@@ -44442,7 +44461,7 @@
         <v>34</v>
       </c>
       <c r="B14" s="18" t="str">
-        <f aca="false">IFERROR(INDEX('Auction Log'!$B$5:$B$304,MATCH(A14,'Auction Log'!$F$5:$F$304,0)),"")</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Auction Log'!$F$5:$F$304=A14)*('Auction Log'!$D$5:$D$304="ME")),'Auction Log'!$B$5:$B$304),"")</f>
         <v/>
       </c>
       <c r="C14" s="18" t="str">
@@ -44450,7 +44469,7 @@
         <v/>
       </c>
       <c r="D14" s="19" t="str">
-        <f aca="false">IFERROR(INDEX('Auction Log'!$E$5:$E$304,MATCH(A14,'Auction Log'!$F$5:$F$304,0)),"")</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Auction Log'!$F$5:$F$304=A14)*('Auction Log'!$D$5:$D$304="ME")),'Auction Log'!$E$5:$E$304),"")</f>
         <v/>
       </c>
       <c r="E14" s="18" t="str">
@@ -44483,7 +44502,7 @@
         <v>37</v>
       </c>
       <c r="B15" s="18" t="str">
-        <f aca="false">IFERROR(INDEX('Auction Log'!$B$5:$B$304,MATCH(A15,'Auction Log'!$F$5:$F$304,0)),"")</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Auction Log'!$F$5:$F$304=A15)*('Auction Log'!$D$5:$D$304="ME")),'Auction Log'!$B$5:$B$304),"")</f>
         <v/>
       </c>
       <c r="C15" s="18" t="str">
@@ -44491,7 +44510,7 @@
         <v/>
       </c>
       <c r="D15" s="19" t="str">
-        <f aca="false">IFERROR(INDEX('Auction Log'!$E$5:$E$304,MATCH(A15,'Auction Log'!$F$5:$F$304,0)),"")</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Auction Log'!$F$5:$F$304=A15)*('Auction Log'!$D$5:$D$304="ME")),'Auction Log'!$E$5:$E$304),"")</f>
         <v/>
       </c>
       <c r="E15" s="18" t="str">
@@ -44524,7 +44543,7 @@
         <v>508</v>
       </c>
       <c r="B16" s="18" t="str">
-        <f aca="false">IFERROR(INDEX('Auction Log'!$B$5:$B$304,MATCH(A16,'Auction Log'!$F$5:$F$304,0)),"")</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Auction Log'!$F$5:$F$304=A16)*('Auction Log'!$D$5:$D$304="ME")),'Auction Log'!$B$5:$B$304),"")</f>
         <v/>
       </c>
       <c r="C16" s="18" t="str">
@@ -44532,7 +44551,7 @@
         <v/>
       </c>
       <c r="D16" s="19" t="str">
-        <f aca="false">IFERROR(INDEX('Auction Log'!$E$5:$E$304,MATCH(A16,'Auction Log'!$F$5:$F$304,0)),"")</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Auction Log'!$F$5:$F$304=A16)*('Auction Log'!$D$5:$D$304="ME")),'Auction Log'!$E$5:$E$304),"")</f>
         <v/>
       </c>
       <c r="E16" s="18" t="str">
@@ -44565,7 +44584,7 @@
         <v>509</v>
       </c>
       <c r="B17" s="18" t="str">
-        <f aca="false">IFERROR(INDEX('Auction Log'!$B$5:$B$304,MATCH(A17,'Auction Log'!$F$5:$F$304,0)),"")</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Auction Log'!$F$5:$F$304=A17)*('Auction Log'!$D$5:$D$304="ME")),'Auction Log'!$B$5:$B$304),"")</f>
         <v/>
       </c>
       <c r="C17" s="18" t="str">
@@ -44573,7 +44592,7 @@
         <v/>
       </c>
       <c r="D17" s="19" t="str">
-        <f aca="false">IFERROR(INDEX('Auction Log'!$E$5:$E$304,MATCH(A17,'Auction Log'!$F$5:$F$304,0)),"")</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Auction Log'!$F$5:$F$304=A17)*('Auction Log'!$D$5:$D$304="ME")),'Auction Log'!$E$5:$E$304),"")</f>
         <v/>
       </c>
       <c r="E17" s="18" t="str">
@@ -44606,7 +44625,7 @@
         <v>510</v>
       </c>
       <c r="B18" s="18" t="str">
-        <f aca="false">IFERROR(INDEX('Auction Log'!$B$5:$B$304,MATCH(A18,'Auction Log'!$F$5:$F$304,0)),"")</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Auction Log'!$F$5:$F$304=A18)*('Auction Log'!$D$5:$D$304="ME")),'Auction Log'!$B$5:$B$304),"")</f>
         <v/>
       </c>
       <c r="C18" s="18" t="str">
@@ -44614,7 +44633,7 @@
         <v/>
       </c>
       <c r="D18" s="19" t="str">
-        <f aca="false">IFERROR(INDEX('Auction Log'!$E$5:$E$304,MATCH(A18,'Auction Log'!$F$5:$F$304,0)),"")</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Auction Log'!$F$5:$F$304=A18)*('Auction Log'!$D$5:$D$304="ME")),'Auction Log'!$E$5:$E$304),"")</f>
         <v/>
       </c>
       <c r="E18" s="18" t="str">
@@ -44647,7 +44666,7 @@
         <v>511</v>
       </c>
       <c r="B19" s="18" t="str">
-        <f aca="false">IFERROR(INDEX('Auction Log'!$B$5:$B$304,MATCH(A19,'Auction Log'!$F$5:$F$304,0)),"")</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Auction Log'!$F$5:$F$304=A19)*('Auction Log'!$D$5:$D$304="ME")),'Auction Log'!$B$5:$B$304),"")</f>
         <v/>
       </c>
       <c r="C19" s="18" t="str">
@@ -44655,7 +44674,7 @@
         <v/>
       </c>
       <c r="D19" s="19" t="str">
-        <f aca="false">IFERROR(INDEX('Auction Log'!$E$5:$E$304,MATCH(A19,'Auction Log'!$F$5:$F$304,0)),"")</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Auction Log'!$F$5:$F$304=A19)*('Auction Log'!$D$5:$D$304="ME")),'Auction Log'!$E$5:$E$304),"")</f>
         <v/>
       </c>
       <c r="E19" s="18" t="str">
@@ -44688,7 +44707,7 @@
         <v>512</v>
       </c>
       <c r="B20" s="18" t="str">
-        <f aca="false">IFERROR(INDEX('Auction Log'!$B$5:$B$304,MATCH(A20,'Auction Log'!$F$5:$F$304,0)),"")</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Auction Log'!$F$5:$F$304=A20)*('Auction Log'!$D$5:$D$304="ME")),'Auction Log'!$B$5:$B$304),"")</f>
         <v/>
       </c>
       <c r="C20" s="18" t="str">
@@ -44696,7 +44715,7 @@
         <v/>
       </c>
       <c r="D20" s="19" t="str">
-        <f aca="false">IFERROR(INDEX('Auction Log'!$E$5:$E$304,MATCH(A20,'Auction Log'!$F$5:$F$304,0)),"")</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Auction Log'!$F$5:$F$304=A20)*('Auction Log'!$D$5:$D$304="ME")),'Auction Log'!$E$5:$E$304),"")</f>
         <v/>
       </c>
       <c r="E20" s="18" t="str">
@@ -44729,7 +44748,7 @@
         <v>513</v>
       </c>
       <c r="B21" s="37" t="str">
-        <f aca="false">IFERROR(INDEX('Auction Log'!$B$5:$B$304,MATCH(A21,'Auction Log'!$F$5:$F$304,0)),"")</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Auction Log'!$F$5:$F$304=A21)*('Auction Log'!$D$5:$D$304="ME")),'Auction Log'!$B$5:$B$304),"")</f>
         <v/>
       </c>
       <c r="C21" s="37" t="str">
@@ -44737,7 +44756,7 @@
         <v/>
       </c>
       <c r="D21" s="38" t="str">
-        <f aca="false">IFERROR(INDEX('Auction Log'!$E$5:$E$304,MATCH(A21,'Auction Log'!$F$5:$F$304,0)),"")</f>
+        <f aca="false">IFERROR(LOOKUP(2,1/(('Auction Log'!$F$5:$F$304=A21)*('Auction Log'!$D$5:$D$304="ME")),'Auction Log'!$E$5:$E$304),"")</f>
         <v/>
       </c>
       <c r="E21" s="37" t="str">

</xml_diff>

<commit_message>
data: refresh pre-draft injury notes
</commit_message>
<xml_diff>
--- a/Draft_Command_Center_DRAFT_DAY.xlsx
+++ b/Draft_Command_Center_DRAFT_DAY.xlsx
@@ -107,7 +107,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2027" uniqueCount="678">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="679" uniqueCount="679">
   <si>
     <t xml:space="preserve">AMERESCO'S BEST — 2026 DRAFT HQ v2</t>
   </si>
@@ -433,7 +433,7 @@
     <t xml:space="preserve">DRAIN</t>
   </si>
   <si>
-    <t xml:space="preserve">Groin - may return to practice the week of 8/24</t>
+    <t>Groin - still questionable; was not practicing as of 8/24 (ESPN 8/26). Discount only — no smash at full Target.</t>
   </si>
   <si>
     <t xml:space="preserve">Amon-Ra St. Brown</t>
@@ -547,7 +547,7 @@
     <t xml:space="preserve">Ashton Jeanty</t>
   </si>
   <si>
-    <t xml:space="preserve">Ankle - diagnosed as a sprain with an unknown timetable for return but not considered a long-term injury (8/23)</t>
+    <t>Ankle - Raiders optimistic 'more low than high' sprain, not long-term (Rapoport 8/25 via ESPN). Buyable near Target; not a healthy stud.</t>
   </si>
   <si>
     <t xml:space="preserve">Garrett Wilson</t>
@@ -562,7 +562,7 @@
     <t xml:space="preserve">NYG</t>
   </si>
   <si>
-    <t xml:space="preserve">Knee - could be out of his non-contact jersey at some point the week of (8/24)</t>
+    <t>Knee - still on limited/red-jersey path as of 8/23 (ESPN). Cap at Target; do not chase.</t>
   </si>
   <si>
     <t xml:space="preserve">Zay Flowers</t>
@@ -589,13 +589,13 @@
     <t xml:space="preserve">Jeremiyah Love</t>
   </si>
   <si>
-    <t xml:space="preserve">High ankle sprain - team is hopeful he will be back by Week 1, but timetable uncertain (8/24)</t>
+    <t>High ankle - light agility only 8/26; est. return Sep 13 (ESPN). Week 1 risk real — fade unless steal.</t>
   </si>
   <si>
     <t xml:space="preserve">Breece Hall</t>
   </si>
   <si>
-    <t xml:space="preserve">Groin - will be sidelined for two to three weeks (8/19)</t>
+    <t>Groin - side agility only 8/24; earlier 2–3 week miss outlook (ESPN). Discount only — early-season hole.</t>
   </si>
   <si>
     <t xml:space="preserve">Javonte Williams</t>
@@ -631,7 +631,7 @@
     <t xml:space="preserve">TB</t>
   </si>
   <si>
-    <t xml:space="preserve">Toe - considered "day-to-day, week-to-week" according to HC; Week 1 status is unclear (8/19)</t>
+    <t>Toe - not participating in practice as of 8/25 (ESPN). Soft pass / require big discount.</t>
   </si>
   <si>
     <t xml:space="preserve">Bucky Irving</t>
@@ -679,19 +679,19 @@
     <t xml:space="preserve">Luther Burden III</t>
   </si>
   <si>
-    <t xml:space="preserve">Groin - will 'hopefully' be ready by the start of the season (8/24)</t>
+    <t>Groin - returned to practice 8/26 but individuals only (ESPN).</t>
   </si>
   <si>
     <t xml:space="preserve">Tyler Warren</t>
   </si>
   <si>
-    <t xml:space="preserve">Groin - expected to miss a week but status for Week 1 is not in danger (8/24)</t>
+    <t>Groin - may sit practice this week but staff preparing him for opener (8/25 via ESPN). Week 1 intent intact.</t>
   </si>
   <si>
     <t xml:space="preserve">Mike Evans</t>
   </si>
   <si>
-    <t xml:space="preserve">Quadriceps - took part in team drills on 8/22</t>
+    <t>Groin - not practicing 8/25 (ESPN). NEW caution vs older quad note — do not pay healthy price.</t>
   </si>
   <si>
     <t xml:space="preserve">Bhayshul Tuten</t>
@@ -724,7 +724,7 @@
     <t xml:space="preserve">PIT</t>
   </si>
   <si>
-    <t xml:space="preserve">Undisclosed - says he is 'fine' and isn't concerned about Week 1 status (8/21)</t>
+    <t>Undisclosed - returned to practice 8/24 after sidelined since 8/8 (ESPN).</t>
   </si>
   <si>
     <t xml:space="preserve">Courtland Sutton</t>
@@ -799,7 +799,7 @@
     <t xml:space="preserve">Sam LaPorta</t>
   </si>
   <si>
-    <t xml:space="preserve">Hip injury - uncertain status for Week 1 (8/24)</t>
+    <t>Hip - returned to practice 8/25 (ESPN). Prior 'uncertain' note stale; OK near Target.</t>
   </si>
   <si>
     <t xml:space="preserve">Jonathon Brooks</t>
@@ -817,13 +817,13 @@
     <t xml:space="preserve">George Kittle</t>
   </si>
   <si>
-    <t xml:space="preserve">Achilles - cleared from PUP list on 8/23; looking good to possibly play in Week 1 (8/24)</t>
+    <t>Achilles - activated from PUP 8/23 (ESPN). Fine as cheap TE upside.</t>
   </si>
   <si>
     <t xml:space="preserve">Tucker Kraft</t>
   </si>
   <si>
-    <t xml:space="preserve">Knee - said he expects the Packers to limit his reps "probably until halfway through the season" (8/19)</t>
+    <t>Knee - participating in team drills 8/26 (ESPN). Less dire than prior half-season limit comment.</t>
   </si>
   <si>
     <t xml:space="preserve">Josh Downs</t>
@@ -853,13 +853,13 @@
     <t xml:space="preserve">Chuba Hubbard</t>
   </si>
   <si>
-    <t xml:space="preserve">Hamstring - considered week-to-week but expected to play in Week 1 (8/24)</t>
+    <t>Hamstring - remains on track for Week 1 (8/24 via ESPN).</t>
   </si>
   <si>
     <t xml:space="preserve">Patrick Mahomes II</t>
   </si>
   <si>
-    <t xml:space="preserve">Knee (ACL) - says he is "extremely confident" he will be available in Week 1 (8/24)</t>
+    <t>Knee (ACL) - 'extremely confident' for Week 1 (8/22 via ESPN). Cheap QB plan still OK.</t>
   </si>
   <si>
     <t xml:space="preserve">Kenny Gainwell</t>
@@ -1000,7 +1000,7 @@
     <t xml:space="preserve">Zach Charbonnet</t>
   </si>
   <si>
-    <t xml:space="preserve">Knee - remains in recovery mode (8/24)</t>
+    <t>Knee - Out / active PUP as of mid-Aug (ESPN). Skip unless $1 lottery.</t>
   </si>
   <si>
     <t xml:space="preserve">Brenton Strange</t>
@@ -1018,7 +1018,7 @@
     <t xml:space="preserve">Alvin Kamara</t>
   </si>
   <si>
-    <t xml:space="preserve">MCL sprain - out at least one month; Week 1 availability in jeopardy (8/24)</t>
+    <t>MCL sprain - out at least ~1 month; Week 1 in jeopardy (Schefter 8/19 via ESPN). Bench dart only.</t>
   </si>
   <si>
     <t xml:space="preserve">Hunter Henry</t>
@@ -1090,7 +1090,7 @@
     <t xml:space="preserve">Jalen McMillan</t>
   </si>
   <si>
-    <t xml:space="preserve">Knee - has returned to practice but HC says he will be "eased back into action" (8/24)</t>
+    <t>Knee - did not travel to 8/26 joint practice (ESPN). Elevated caution.</t>
   </si>
   <si>
     <t xml:space="preserve">Tre' Harris</t>
@@ -2141,6 +2141,9 @@
   </si>
   <si>
     <t xml:space="preserve">MY HAUL</t>
+  </si>
+  <si>
+    <t>Foot - too early to tell on Week 1 availability (coach 8/26 via ESPN).</t>
   </si>
 </sst>
 </file>
@@ -6309,7 +6312,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
@@ -24815,7 +24818,9 @@
       <c r="T208" s="18" t="s">
         <v>291</v>
       </c>
-      <c r="U208" s="32"/>
+      <c r="U208" s="32" t="s">
+        <v>678</v>
+      </c>
       <c r="V208" s="19" t="str">
         <f aca="false">IF(E208="","",R208-E208)</f>
         <v/>
@@ -45001,7 +45006,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>

</xml_diff>